<commit_message>
fix: fixed login flow
</commit_message>
<xml_diff>
--- a/data/candidates.xlsx
+++ b/data/candidates.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="171">
   <si>
     <t>candidateId</t>
   </si>
@@ -411,6 +411,66 @@
   </si>
   <si>
     <t>1a153fcd672c95cb</t>
+  </si>
+  <si>
+    <t>Ravikant Shahi</t>
+  </si>
+  <si>
+    <t>shahi.ravikant5661@gmail.com</t>
+  </si>
+  <si>
+    <t>+91 6207929187</t>
+  </si>
+  <si>
+    <t>Ravikant Shahi is a Backend Developer with practical industry experience building scalable RESTful APIs, relational database schemas, and external API integrations using Node.js, Express.js, and MySQL. Demonstrates strong competency in query optimization, OAuth 2.0, and RBAC.</t>
+  </si>
+  <si>
+    <t>ravikant_backend_2years.pdf</t>
+  </si>
+  <si>
+    <t>1a15819a2708bad2</t>
+  </si>
+  <si>
+    <t>Ravi Singh</t>
+  </si>
+  <si>
+    <t>ravisingh.qa@email.com</t>
+  </si>
+  <si>
+    <t>+91 XXXXXXXXXX</t>
+  </si>
+  <si>
+    <t>QA Automation Engineer</t>
+  </si>
+  <si>
+    <t>Ravi Singh is an experienced QA Automation Engineer with strong backend and API automation expertise across Python, JavaScript, RestAssured, and Postman/Newman, alongside CI/CD pipeline integration via GitHub Actions and Jenkins.</t>
+  </si>
+  <si>
+    <t>Cover Letter Doc in Blue White Clean Style.pdf</t>
+  </si>
+  <si>
+    <t>1a158431e57f9b2a</t>
+  </si>
+  <si>
+    <t>Isabel Mercado</t>
+  </si>
+  <si>
+    <t>hello@reallygreatsite.com</t>
+  </si>
+  <si>
+    <t>123-456-7890</t>
+  </si>
+  <si>
+    <t>Digital Marketer</t>
+  </si>
+  <si>
+    <t>Isabel Mercado submitted an application indicating digital marketing leadership experience in the cover email, but the attached resume contains placeholder (Lorem ipsum) text under job descriptions and primarily lists Product Design Manager roles. Key digital marketing competencies such as SEO, Google Analytics, and paid ad management lack substantiation.</t>
+  </si>
+  <si>
+    <t>Minimalist CV Resume.pdf</t>
+  </si>
+  <si>
+    <t>1a15867e0c600589</t>
   </si>
   <si>
     <t>Section</t>
@@ -874,7 +934,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB17"/>
+  <dimension ref="A1:AB20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1610,7 +1670,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>15</v>
       </c>
@@ -1649,6 +1709,129 @@
       </c>
       <c r="M17" t="s">
         <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>18</v>
+      </c>
+      <c r="B18" t="s">
+        <v>133</v>
+      </c>
+      <c r="C18" t="s">
+        <v>134</v>
+      </c>
+      <c r="D18" t="s">
+        <v>135</v>
+      </c>
+      <c r="E18" t="s">
+        <v>115</v>
+      </c>
+      <c r="F18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G18" t="s">
+        <v>18</v>
+      </c>
+      <c r="H18" t="s">
+        <v>19</v>
+      </c>
+      <c r="I18">
+        <v>86</v>
+      </c>
+      <c r="J18" t="s">
+        <v>136</v>
+      </c>
+      <c r="K18" t="s">
+        <v>137</v>
+      </c>
+      <c r="L18" t="s">
+        <v>138</v>
+      </c>
+      <c r="M18" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>19</v>
+      </c>
+      <c r="B19" t="s">
+        <v>139</v>
+      </c>
+      <c r="C19" t="s">
+        <v>140</v>
+      </c>
+      <c r="D19" t="s">
+        <v>141</v>
+      </c>
+      <c r="E19" t="s">
+        <v>142</v>
+      </c>
+      <c r="F19" t="s">
+        <v>17</v>
+      </c>
+      <c r="G19" t="s">
+        <v>18</v>
+      </c>
+      <c r="H19" t="s">
+        <v>29</v>
+      </c>
+      <c r="I19">
+        <v>84</v>
+      </c>
+      <c r="J19" t="s">
+        <v>143</v>
+      </c>
+      <c r="K19" t="s">
+        <v>144</v>
+      </c>
+      <c r="L19" t="s">
+        <v>145</v>
+      </c>
+      <c r="M19" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>20</v>
+      </c>
+      <c r="B20" t="s">
+        <v>146</v>
+      </c>
+      <c r="C20" t="s">
+        <v>147</v>
+      </c>
+      <c r="D20" t="s">
+        <v>148</v>
+      </c>
+      <c r="E20" t="s">
+        <v>149</v>
+      </c>
+      <c r="F20" t="s">
+        <v>74</v>
+      </c>
+      <c r="G20" t="s">
+        <v>18</v>
+      </c>
+      <c r="H20" t="s">
+        <v>29</v>
+      </c>
+      <c r="I20">
+        <v>15</v>
+      </c>
+      <c r="J20" t="s">
+        <v>150</v>
+      </c>
+      <c r="K20" t="s">
+        <v>151</v>
+      </c>
+      <c r="L20" t="s">
+        <v>152</v>
+      </c>
+      <c r="M20" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -1668,74 +1851,74 @@
   <sheetData>
     <row r="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>133</v>
+        <v>153</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>134</v>
+        <v>154</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>135</v>
+        <v>155</v>
       </c>
       <c r="B2" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>137</v>
+        <v>157</v>
       </c>
       <c r="B3" t="s">
-        <v>138</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>139</v>
+        <v>159</v>
       </c>
       <c r="B4" t="s">
-        <v>140</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>141</v>
+        <v>161</v>
       </c>
       <c r="B5" t="s">
-        <v>142</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>143</v>
+        <v>163</v>
       </c>
       <c r="B6" t="s">
-        <v>144</v>
+        <v>164</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>145</v>
+        <v>165</v>
       </c>
       <c r="B7" t="s">
-        <v>146</v>
+        <v>166</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>147</v>
+        <v>167</v>
       </c>
       <c r="B8" t="s">
-        <v>148</v>
+        <v>168</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>149</v>
+        <v>169</v>
       </c>
       <c r="B9" t="s">
-        <v>150</v>
+        <v>170</v>
       </c>
     </row>
   </sheetData>

</xml_diff>